<commit_message>
version updated screen success
</commit_message>
<xml_diff>
--- a/Screener/ScreenResult/ScreenResult.xlsx
+++ b/Screener/ScreenResult/ScreenResult.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>Symbol</t>
   </si>
@@ -79,22 +79,34 @@
     <t>ELF</t>
   </si>
   <si>
+    <t>HTGC</t>
+  </si>
+  <si>
     <t>Technology</t>
   </si>
   <si>
     <t>Consumer Defensive</t>
   </si>
   <si>
+    <t>Financial Services</t>
+  </si>
+  <si>
     <t>Computer Hardware</t>
   </si>
   <si>
     <t>Household &amp; Personal Products</t>
   </si>
   <si>
+    <t>Asset Management</t>
+  </si>
+  <si>
     <t>2007-03-29</t>
   </si>
   <si>
     <t>2016-09-22</t>
+  </si>
+  <si>
+    <t>2005-06-09</t>
   </si>
 </sst>
 </file>
@@ -452,7 +464,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S3"/>
+  <dimension ref="A1:S4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:19">
@@ -519,46 +531,46 @@
         <v>19</v>
       </c>
       <c r="B2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D2" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E2">
-        <v>866.1199951171875</v>
+        <v>1085.415649414062</v>
       </c>
       <c r="F2">
-        <v>14772216.66666667</v>
+        <v>14819195.63333333</v>
       </c>
       <c r="G2">
-        <v>528.3253985595703</v>
+        <v>637.4673095703125</v>
       </c>
       <c r="H2">
-        <v>358.9864657592773</v>
+        <v>394.1328362019857</v>
       </c>
       <c r="I2">
-        <v>329.163299331665</v>
+        <v>361.5986769866943</v>
       </c>
       <c r="J2">
-        <v>262.5819494247436</v>
+        <v>282.0150992584229</v>
       </c>
       <c r="K2">
-        <v>89.27999877929688</v>
+        <v>91.75</v>
       </c>
       <c r="L2">
-        <v>1004</v>
+        <v>1159.760009765625</v>
       </c>
       <c r="M2">
-        <v>203.2527010745317</v>
+        <v>323.7422117030001</v>
       </c>
       <c r="N2">
-        <v>785.3316762815909</v>
+        <v>1073.803001065657</v>
       </c>
       <c r="O2">
-        <v>441.3718115269876</v>
+        <v>557.7662072666031</v>
       </c>
       <c r="P2">
         <v>62</v>
@@ -578,46 +590,46 @@
         <v>20</v>
       </c>
       <c r="B3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D3" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E3">
-        <v>208.5299987792969</v>
+        <v>193.6100006103516</v>
       </c>
       <c r="F3">
-        <v>1756746.666666667</v>
+        <v>1440388.8</v>
       </c>
       <c r="G3">
-        <v>162.0811996459961</v>
+        <v>170.4341995239258</v>
       </c>
       <c r="H3">
-        <v>131.8589999389648</v>
+        <v>135.7615998840332</v>
       </c>
       <c r="I3">
-        <v>125.4374499511719</v>
+        <v>129.5238999176025</v>
       </c>
       <c r="J3">
-        <v>116.7663999557495</v>
+        <v>119.4194500350952</v>
       </c>
       <c r="K3">
-        <v>69.56999969482422</v>
+        <v>72.01999664306641</v>
       </c>
       <c r="L3">
-        <v>208.5299987792969</v>
+        <v>217.3999938964844</v>
       </c>
       <c r="M3">
-        <v>76.4362420439728</v>
+        <v>52.56895057709545</v>
       </c>
       <c r="N3">
-        <v>177.3374012612904</v>
+        <v>168.828116682495</v>
       </c>
       <c r="O3">
-        <v>197.3505742430945</v>
+        <v>179.6599058749279</v>
       </c>
       <c r="P3">
         <v>35</v>
@@ -630,6 +642,65 @@
       </c>
       <c r="S3">
         <v>25.889</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19">
+      <c r="A4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E4">
+        <v>18.16500091552734</v>
+      </c>
+      <c r="F4">
+        <v>1052424.7</v>
+      </c>
+      <c r="G4">
+        <v>17.23304351806641</v>
+      </c>
+      <c r="H4">
+        <v>15.93628141403198</v>
+      </c>
+      <c r="I4">
+        <v>15.47844623088837</v>
+      </c>
+      <c r="J4">
+        <v>14.88064412593842</v>
+      </c>
+      <c r="K4">
+        <v>10.24463176727295</v>
+      </c>
+      <c r="L4">
+        <v>18.39999961853027</v>
+      </c>
+      <c r="M4">
+        <v>21.68225148065475</v>
+      </c>
+      <c r="N4">
+        <v>71.52562697174625</v>
+      </c>
+      <c r="O4">
+        <v>124.5966768115443</v>
+      </c>
+      <c r="P4">
+        <v>66</v>
+      </c>
+      <c r="Q4">
+        <v>192</v>
+      </c>
+      <c r="R4">
+        <v>171</v>
+      </c>
+      <c r="S4">
+        <v>21.065001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update new method to get ticker
</commit_message>
<xml_diff>
--- a/Screener/ScreenResult/ScreenResult.xlsx
+++ b/Screener/ScreenResult/ScreenResult.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="134">
   <si>
     <t>Symbol</t>
   </si>
@@ -88,108 +88,114 @@
     <t>NVDA</t>
   </si>
   <si>
+    <t>POWL</t>
+  </si>
+  <si>
     <t>MMYT</t>
   </si>
   <si>
+    <t>ELF</t>
+  </si>
+  <si>
     <t>STRL</t>
   </si>
   <si>
-    <t>ELF</t>
-  </si>
-  <si>
     <t>UBER</t>
   </si>
   <si>
     <t>VIST</t>
   </si>
   <si>
+    <t>AEO</t>
+  </si>
+  <si>
     <t>AROC</t>
   </si>
   <si>
-    <t>AEO</t>
+    <t>ETN</t>
+  </si>
+  <si>
+    <t>ROAD</t>
   </si>
   <si>
     <t>WMS</t>
   </si>
   <si>
+    <t>MCY</t>
+  </si>
+  <si>
     <t>WFRD</t>
   </si>
   <si>
-    <t>ETN</t>
-  </si>
-  <si>
-    <t>ROAD</t>
-  </si>
-  <si>
-    <t>MCY</t>
+    <t>PCAR</t>
+  </si>
+  <si>
+    <t>ASML</t>
+  </si>
+  <si>
+    <t>ALSN</t>
   </si>
   <si>
     <t>DVA</t>
   </si>
   <si>
-    <t>ALSN</t>
-  </si>
-  <si>
-    <t>ASML</t>
-  </si>
-  <si>
-    <t>PCAR</t>
+    <t>MLM</t>
+  </si>
+  <si>
+    <t>SAP</t>
+  </si>
+  <si>
+    <t>PH</t>
   </si>
   <si>
     <t>HWM</t>
   </si>
   <si>
-    <t>MLM</t>
-  </si>
-  <si>
-    <t>PH</t>
+    <t>HUBB</t>
   </si>
   <si>
     <t>AMZN</t>
   </si>
   <si>
-    <t>SAP</t>
+    <t>NTAP</t>
   </si>
   <si>
     <t>HIG</t>
   </si>
   <si>
-    <t>HUBB</t>
-  </si>
-  <si>
-    <t>NTAP</t>
-  </si>
-  <si>
     <t>NOW</t>
   </si>
   <si>
+    <t>JPM</t>
+  </si>
+  <si>
+    <t>GRMN</t>
+  </si>
+  <si>
+    <t>MANH</t>
+  </si>
+  <si>
     <t>SHOP</t>
   </si>
   <si>
-    <t>GRMN</t>
-  </si>
-  <si>
-    <t>JPM</t>
-  </si>
-  <si>
-    <t>MANH</t>
-  </si>
-  <si>
     <t>MOH</t>
   </si>
   <si>
+    <t>SNPS</t>
+  </si>
+  <si>
     <t>BRO</t>
   </si>
   <si>
-    <t>SNPS</t>
+    <t>LPG</t>
+  </si>
+  <si>
+    <t>ZWS</t>
   </si>
   <si>
     <t>WWD</t>
   </si>
   <si>
-    <t>ZWS</t>
-  </si>
-  <si>
     <t>Technology</t>
   </si>
   <si>
@@ -232,64 +238,67 @@
     <t>Travel Services</t>
   </si>
   <si>
+    <t>Household &amp; Personal Products</t>
+  </si>
+  <si>
     <t>Engineering &amp; Construction</t>
   </si>
   <si>
-    <t>Household &amp; Personal Products</t>
-  </si>
-  <si>
     <t>Software—Application</t>
   </si>
   <si>
     <t>Oil &amp; Gas E&amp;P</t>
   </si>
   <si>
+    <t>Apparel Retail</t>
+  </si>
+  <si>
     <t>Oil &amp; Gas Equipment &amp; Services</t>
   </si>
   <si>
-    <t>Apparel Retail</t>
+    <t>Specialty Industrial Machinery</t>
   </si>
   <si>
     <t>Building Products &amp; Equipment</t>
   </si>
   <si>
-    <t>Specialty Industrial Machinery</t>
-  </si>
-  <si>
     <t>Insurance—Property &amp; Casualty</t>
   </si>
   <si>
+    <t>Farm &amp; Heavy Construction Machinery</t>
+  </si>
+  <si>
+    <t>Semiconductor Equipment &amp; Materials</t>
+  </si>
+  <si>
     <t>Medical Care Facilities</t>
   </si>
   <si>
-    <t>Semiconductor Equipment &amp; Materials</t>
-  </si>
-  <si>
-    <t>Farm &amp; Heavy Construction Machinery</t>
+    <t>Building Materials</t>
   </si>
   <si>
     <t>Aerospace &amp; Defense</t>
   </si>
   <si>
-    <t>Building Materials</t>
-  </si>
-  <si>
     <t>Internet Retail</t>
   </si>
   <si>
+    <t>Banks—Diversified</t>
+  </si>
+  <si>
     <t>Scientific &amp; Technical Instruments</t>
   </si>
   <si>
-    <t>Banks—Diversified</t>
-  </si>
-  <si>
     <t>Healthcare Plans</t>
   </si>
   <si>
+    <t>Software—Infrastructure</t>
+  </si>
+  <si>
     <t>Insurance Brokers</t>
   </si>
   <si>
-    <t>Software—Infrastructure</t>
+    <t>Oil &amp; Gas Midstream</t>
   </si>
   <si>
     <t>Pollution &amp; Treatment Controls</t>
@@ -310,100 +319,103 @@
     <t>1999-01-22</t>
   </si>
   <si>
+    <t>1980-03-17</t>
+  </si>
+  <si>
     <t>2010-08-12</t>
   </si>
   <si>
+    <t>2016-09-22</t>
+  </si>
+  <si>
     <t>1991-07-12</t>
   </si>
   <si>
-    <t>2016-09-22</t>
-  </si>
-  <si>
     <t>2019-05-10</t>
   </si>
   <si>
     <t>2019-07-26</t>
   </si>
   <si>
+    <t>1994-04-14</t>
+  </si>
+  <si>
     <t>2007-08-21</t>
   </si>
   <si>
-    <t>1994-04-14</t>
+    <t>1972-06-01</t>
+  </si>
+  <si>
+    <t>2018-05-04</t>
   </si>
   <si>
     <t>2014-07-25</t>
   </si>
   <si>
+    <t>1985-11-20</t>
+  </si>
+  <si>
     <t>2021-01-04</t>
   </si>
   <si>
-    <t>1972-06-01</t>
-  </si>
-  <si>
-    <t>2018-05-04</t>
-  </si>
-  <si>
-    <t>1985-11-20</t>
+    <t>1995-03-15</t>
+  </si>
+  <si>
+    <t>2012-03-15</t>
   </si>
   <si>
     <t>1995-10-31</t>
   </si>
   <si>
-    <t>2012-03-15</t>
-  </si>
-  <si>
-    <t>1995-03-15</t>
-  </si>
-  <si>
-    <t>1980-03-17</t>
+    <t>1994-02-17</t>
+  </si>
+  <si>
+    <t>1995-09-18</t>
   </si>
   <si>
     <t>2016-11-01</t>
   </si>
   <si>
-    <t>1994-02-17</t>
+    <t>1972-06-05</t>
   </si>
   <si>
     <t>1997-05-15</t>
   </si>
   <si>
-    <t>1995-09-18</t>
+    <t>1995-11-21</t>
   </si>
   <si>
     <t>1995-12-15</t>
   </si>
   <si>
-    <t>1972-06-05</t>
-  </si>
-  <si>
-    <t>1995-11-21</t>
-  </si>
-  <si>
     <t>2012-06-29</t>
   </si>
   <si>
+    <t>2000-12-08</t>
+  </si>
+  <si>
+    <t>1998-04-23</t>
+  </si>
+  <si>
     <t>2015-05-20</t>
   </si>
   <si>
-    <t>2000-12-08</t>
-  </si>
-  <si>
-    <t>1998-04-23</t>
-  </si>
-  <si>
     <t>2003-07-02</t>
   </si>
   <si>
+    <t>1992-02-26</t>
+  </si>
+  <si>
     <t>1981-02-11</t>
   </si>
   <si>
-    <t>1992-02-26</t>
+    <t>2014-05-08</t>
+  </si>
+  <si>
+    <t>2012-03-29</t>
   </si>
   <si>
     <t>1994-04-04</t>
-  </si>
-  <si>
-    <t>2012-03-29</t>
   </si>
 </sst>
 </file>
@@ -761,7 +773,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S40"/>
+  <dimension ref="A1:S42"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:19">
@@ -828,31 +840,31 @@
         <v>19</v>
       </c>
       <c r="B2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D2" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E2">
-        <v>896.469970703125</v>
+        <v>971.6099853515625</v>
       </c>
       <c r="F2">
-        <v>13593680</v>
+        <v>13471650</v>
       </c>
       <c r="G2">
-        <v>743.6657916259766</v>
+        <v>756.2233911132812</v>
       </c>
       <c r="H2">
-        <v>429.6053972371419</v>
+        <v>434.3912638346354</v>
       </c>
       <c r="I2">
-        <v>390.8399977111816</v>
+        <v>394.5797476196289</v>
       </c>
       <c r="J2">
-        <v>306.99169921875</v>
+        <v>311.1831493377686</v>
       </c>
       <c r="K2">
         <v>93.27999877929688</v>
@@ -861,13 +873,13 @@
         <v>1188.069946289062</v>
       </c>
       <c r="M2">
-        <v>178.2426406499555</v>
+        <v>207.5299037296665</v>
       </c>
       <c r="N2">
-        <v>686.377167283443</v>
+        <v>776.6669397268894</v>
       </c>
       <c r="O2">
-        <v>439.245446730372</v>
+        <v>480.8371576333672</v>
       </c>
       <c r="P2">
         <v>62</v>
@@ -887,46 +899,46 @@
         <v>20</v>
       </c>
       <c r="B3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D3" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E3">
-        <v>77.83999633789062</v>
+        <v>82.11000061035156</v>
       </c>
       <c r="F3">
-        <v>8628510</v>
+        <v>8785383.333333334</v>
       </c>
       <c r="G3">
-        <v>62.18179985046387</v>
+        <v>62.84039985656738</v>
       </c>
       <c r="H3">
-        <v>48.08573331197103</v>
+        <v>48.40819997151693</v>
       </c>
       <c r="I3">
-        <v>42.63484999656677</v>
+        <v>42.94505000114441</v>
       </c>
       <c r="J3">
-        <v>37.25550003528595</v>
+        <v>37.49510004520416</v>
       </c>
       <c r="K3">
         <v>12.18000030517578</v>
       </c>
       <c r="L3">
-        <v>77.83999633789062</v>
+        <v>82.11000061035156</v>
       </c>
       <c r="M3">
-        <v>62.84518322238657</v>
+        <v>66.82242700923402</v>
       </c>
       <c r="N3">
-        <v>488.3597810369461</v>
+        <v>527.272724623448</v>
       </c>
       <c r="O3">
-        <v>293.0237150315805</v>
+        <v>305.5843918862921</v>
       </c>
       <c r="P3">
         <v>857</v>
@@ -946,46 +958,46 @@
         <v>21</v>
       </c>
       <c r="B4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D4" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="E4">
-        <v>99</v>
+        <v>102.6999969482422</v>
       </c>
       <c r="F4">
-        <v>1092100</v>
+        <v>1133660</v>
       </c>
       <c r="G4">
-        <v>76.6597999572754</v>
+        <v>77.49779991149903</v>
       </c>
       <c r="H4">
-        <v>57.71353329976399</v>
+        <v>58.10626660664877</v>
       </c>
       <c r="I4">
-        <v>52.2904000377655</v>
+        <v>52.65550002098084</v>
       </c>
       <c r="J4">
-        <v>45.77190006256104</v>
+        <v>46.07585007667542</v>
       </c>
       <c r="K4">
         <v>19.5</v>
       </c>
       <c r="L4">
-        <v>99</v>
+        <v>102.6999969482422</v>
       </c>
       <c r="M4">
-        <v>75.59417900754137</v>
+        <v>76.64258346471095</v>
       </c>
       <c r="N4">
-        <v>344.3446900759747</v>
+        <v>371.1009199195274</v>
       </c>
       <c r="O4">
-        <v>269.0828339926385</v>
+        <v>274.0218802161012</v>
       </c>
       <c r="P4">
         <v>80</v>
@@ -1005,31 +1017,31 @@
         <v>22</v>
       </c>
       <c r="B5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D5" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="E5">
-        <v>44.04999923706055</v>
+        <v>47.04999923706055</v>
       </c>
       <c r="F5">
-        <v>2288293.333333333</v>
+        <v>2309246.666666667</v>
       </c>
       <c r="G5">
-        <v>37.94179973602295</v>
+        <v>38.30779972076416</v>
       </c>
       <c r="H5">
-        <v>29.61059992472331</v>
+        <v>29.783733253479</v>
       </c>
       <c r="I5">
-        <v>26.33129990577698</v>
+        <v>26.50139990329743</v>
       </c>
       <c r="J5">
-        <v>23.08064994335174</v>
+        <v>23.23439994335175</v>
       </c>
       <c r="K5">
         <v>10.63000011444092</v>
@@ -1038,13 +1050,13 @@
         <v>47.36999893188477</v>
       </c>
       <c r="M5">
-        <v>49.7789849221528</v>
+        <v>60.14295636839251</v>
       </c>
       <c r="N5">
-        <v>254.0996842678614</v>
+        <v>280.3556966236305</v>
       </c>
       <c r="O5">
-        <v>233.0659722969006</v>
+        <v>246.4525541668191</v>
       </c>
       <c r="P5">
         <v>100</v>
@@ -1064,31 +1076,31 @@
         <v>23</v>
       </c>
       <c r="B6" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D6" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="E6">
-        <v>903.719970703125</v>
+        <v>914.3499755859375</v>
       </c>
       <c r="F6">
-        <v>59481803.33333334</v>
+        <v>59441646.66666666</v>
       </c>
       <c r="G6">
-        <v>724.4649975585937</v>
+        <v>732.1239965820313</v>
       </c>
       <c r="H6">
-        <v>548.7159999593099</v>
+        <v>551.9125998942058</v>
       </c>
       <c r="I6">
-        <v>519.4898001098633</v>
+        <v>522.1030000305176</v>
       </c>
       <c r="J6">
-        <v>466.6388003540039</v>
+        <v>469.1317004394531</v>
       </c>
       <c r="K6">
         <v>262.4100036621094</v>
@@ -1097,13 +1109,13 @@
         <v>926.6900024414062</v>
       </c>
       <c r="M6">
-        <v>80.46608034221714</v>
+        <v>84.32988465347408</v>
       </c>
       <c r="N6">
-        <v>232.3599567988452</v>
+        <v>241.442901680387</v>
       </c>
       <c r="O6">
-        <v>231.1826315040106</v>
+        <v>230.8797040260948</v>
       </c>
       <c r="P6">
         <v>1230</v>
@@ -1123,58 +1135,58 @@
         <v>24</v>
       </c>
       <c r="B7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C7" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D7" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="E7">
-        <v>67.26000213623047</v>
+        <v>142.0500030517578</v>
       </c>
       <c r="F7">
-        <v>807010</v>
+        <v>418110</v>
       </c>
       <c r="G7">
-        <v>56.50439964294434</v>
+        <v>132.3232019042969</v>
       </c>
       <c r="H7">
-        <v>46.28639986673991</v>
+        <v>99.33400075276693</v>
       </c>
       <c r="I7">
-        <v>42.07099989891052</v>
+        <v>90.78020051956177</v>
       </c>
       <c r="J7">
-        <v>38.53859991073608</v>
+        <v>80.2696502494812</v>
       </c>
       <c r="K7">
-        <v>22.51000022888184</v>
+        <v>39.02999877929688</v>
       </c>
       <c r="L7">
-        <v>67.26000213623047</v>
+        <v>185.2400054931641</v>
       </c>
       <c r="M7">
-        <v>43.810137861706</v>
+        <v>47.90712380011208</v>
       </c>
       <c r="N7">
-        <v>176.448838253778</v>
+        <v>244.9490092254905</v>
       </c>
       <c r="O7">
-        <v>202.3363634031878</v>
+        <v>214.4020694163537</v>
       </c>
       <c r="P7">
-        <v>21900</v>
+        <v>1880</v>
       </c>
       <c r="Q7">
-        <v>76</v>
+        <v>291</v>
       </c>
       <c r="R7">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="S7">
-        <v>5.58</v>
+        <v>23.3</v>
       </c>
     </row>
     <row r="8" spans="1:19">
@@ -1182,58 +1194,58 @@
         <v>25</v>
       </c>
       <c r="B8" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C8" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D8" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="E8">
-        <v>109.6900024414062</v>
+        <v>68.52999877929688</v>
       </c>
       <c r="F8">
-        <v>411976.6666666667</v>
+        <v>813840</v>
       </c>
       <c r="G8">
-        <v>89.38920013427735</v>
+        <v>56.97779960632325</v>
       </c>
       <c r="H8">
-        <v>79.18219998677571</v>
+        <v>46.50053319295247</v>
       </c>
       <c r="I8">
-        <v>74.18185001373291</v>
+        <v>42.27559988975525</v>
       </c>
       <c r="J8">
-        <v>68.06524991989136</v>
+        <v>38.70489992141724</v>
       </c>
       <c r="K8">
-        <v>34.63999938964844</v>
+        <v>22.51000022888184</v>
       </c>
       <c r="L8">
-        <v>111.9800033569336</v>
+        <v>68.52999877929688</v>
       </c>
       <c r="M8">
-        <v>39.59022637494638</v>
+        <v>46.24412694556885</v>
       </c>
       <c r="N8">
-        <v>189.4195198554482</v>
+        <v>184.7112573667083</v>
       </c>
       <c r="O8">
-        <v>183.7415512152612</v>
+        <v>203.7549135064658</v>
       </c>
       <c r="P8">
-        <v>307</v>
+        <v>21900</v>
       </c>
       <c r="Q8">
-        <v>28</v>
+        <v>76</v>
       </c>
       <c r="R8">
-        <v>67</v>
+        <v>25</v>
       </c>
       <c r="S8">
-        <v>25.933</v>
+        <v>5.58</v>
       </c>
     </row>
     <row r="9" spans="1:19">
@@ -1241,46 +1253,46 @@
         <v>26</v>
       </c>
       <c r="B9" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C9" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D9" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="E9">
-        <v>200.5399932861328</v>
+        <v>207.3099975585938</v>
       </c>
       <c r="F9">
-        <v>1404836.666666667</v>
+        <v>1310993.333333333</v>
       </c>
       <c r="G9">
-        <v>178.686598815918</v>
+        <v>179.7391989135742</v>
       </c>
       <c r="H9">
-        <v>138.9233996073405</v>
+        <v>139.4420662943522</v>
       </c>
       <c r="I9">
-        <v>132.9602497863769</v>
+        <v>133.4712497711182</v>
       </c>
       <c r="J9">
-        <v>122.1878499984741</v>
+        <v>122.6577499771118</v>
       </c>
       <c r="K9">
-        <v>75.19000244140625</v>
+        <v>78.48000335693359</v>
       </c>
       <c r="L9">
         <v>217.3999938964844</v>
       </c>
       <c r="M9">
-        <v>35.70171534892941</v>
+        <v>35.91424586488115</v>
       </c>
       <c r="N9">
-        <v>166.7109812137708</v>
+        <v>164.1564585767544</v>
       </c>
       <c r="O9">
-        <v>181.5074152704412</v>
+        <v>185.610261162441</v>
       </c>
       <c r="P9">
         <v>35</v>
@@ -1300,58 +1312,58 @@
         <v>27</v>
       </c>
       <c r="B10" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C10" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D10" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="E10">
-        <v>78.63999938964844</v>
+        <v>109.9499969482422</v>
       </c>
       <c r="F10">
-        <v>20411926.66666667</v>
+        <v>414626.6666666667</v>
       </c>
       <c r="G10">
-        <v>72.29660011291504</v>
+        <v>90.04640014648437</v>
       </c>
       <c r="H10">
-        <v>57.79933326721191</v>
+        <v>79.37859998067221</v>
       </c>
       <c r="I10">
-        <v>54.40589994430542</v>
+        <v>74.4820000076294</v>
       </c>
       <c r="J10">
-        <v>50.40714994430542</v>
+        <v>68.27429992675781</v>
       </c>
       <c r="K10">
-        <v>29.59000015258789</v>
+        <v>34.63999938964844</v>
       </c>
       <c r="L10">
-        <v>81.38999938964844</v>
+        <v>111.9800033569336</v>
       </c>
       <c r="M10">
-        <v>27.39348772527062</v>
+        <v>36.44824329833733</v>
       </c>
       <c r="N10">
-        <v>152.2129525976767</v>
+        <v>189.1138587364294</v>
       </c>
       <c r="O10">
-        <v>174.0271967096356</v>
+        <v>181.8059609339164</v>
       </c>
       <c r="P10">
-        <v>128</v>
+        <v>307</v>
       </c>
       <c r="Q10">
-        <v>119</v>
+        <v>28</v>
       </c>
       <c r="R10">
-        <v>15</v>
+        <v>67</v>
       </c>
       <c r="S10">
-        <v>20.353001</v>
+        <v>25.933</v>
       </c>
     </row>
     <row r="11" spans="1:19">
@@ -1359,58 +1371,58 @@
         <v>28</v>
       </c>
       <c r="B11" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C11" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D11" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="E11">
-        <v>42.9900016784668</v>
+        <v>80.25</v>
       </c>
       <c r="F11">
-        <v>567780</v>
+        <v>19506326.66666667</v>
       </c>
       <c r="G11">
-        <v>34.3623999786377</v>
+        <v>72.69560012817382</v>
       </c>
       <c r="H11">
-        <v>30.52693328857422</v>
+        <v>58.04333325703939</v>
       </c>
       <c r="I11">
-        <v>29.08119996070862</v>
+        <v>54.60504995346069</v>
       </c>
       <c r="J11">
-        <v>27.38244996070862</v>
+        <v>50.6085499382019</v>
       </c>
       <c r="K11">
-        <v>16.79000091552734</v>
+        <v>29.59000015258789</v>
       </c>
       <c r="L11">
-        <v>42.9900016784668</v>
+        <v>81.38999938964844</v>
       </c>
       <c r="M11">
-        <v>41.22864955395676</v>
+        <v>29.18544974219168</v>
       </c>
       <c r="N11">
-        <v>150.3785759315265</v>
+        <v>160.9756097560976</v>
       </c>
       <c r="O11">
-        <v>168.86017272672</v>
+        <v>177.9614465006098</v>
       </c>
       <c r="P11">
-        <v>54</v>
+        <v>128</v>
       </c>
       <c r="Q11">
-        <v>407</v>
+        <v>119</v>
       </c>
       <c r="R11">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="S11">
-        <v>37.967</v>
+        <v>20.353001</v>
       </c>
     </row>
     <row r="12" spans="1:19">
@@ -1418,58 +1430,58 @@
         <v>29</v>
       </c>
       <c r="B12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C12" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D12" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="E12">
-        <v>19.29000091552734</v>
+        <v>43.27000045776367</v>
       </c>
       <c r="F12">
-        <v>1408093.333333333</v>
+        <v>578623.3333333334</v>
       </c>
       <c r="G12">
-        <v>16.9820000076294</v>
+        <v>34.63819999694825</v>
       </c>
       <c r="H12">
-        <v>14.68739998499552</v>
+        <v>30.64693328857422</v>
       </c>
       <c r="I12">
-        <v>13.73624998092651</v>
+        <v>29.18744996070862</v>
       </c>
       <c r="J12">
-        <v>12.84669997692108</v>
+        <v>27.46104996681213</v>
       </c>
       <c r="K12">
-        <v>9</v>
+        <v>16.79000091552734</v>
       </c>
       <c r="L12">
-        <v>19.29000091552734</v>
+        <v>43.27000045776367</v>
       </c>
       <c r="M12">
-        <v>24.77361492839578</v>
+        <v>39.71585862807987</v>
       </c>
       <c r="N12">
-        <v>110.1307219418221</v>
+        <v>157.7129130335407</v>
       </c>
       <c r="O12">
-        <v>164.9105355520235</v>
+        <v>170.9056262139584</v>
       </c>
       <c r="P12">
-        <v>657</v>
+        <v>54</v>
       </c>
       <c r="Q12">
-        <v>139</v>
+        <v>407</v>
       </c>
       <c r="R12">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="S12">
-        <v>12.126</v>
+        <v>37.967</v>
       </c>
     </row>
     <row r="13" spans="1:19">
@@ -1477,46 +1489,46 @@
         <v>30</v>
       </c>
       <c r="B13" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C13" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D13" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E13">
-        <v>24.84000015258789</v>
+        <v>25.8799991607666</v>
       </c>
       <c r="F13">
-        <v>4933140</v>
+        <v>5080380</v>
       </c>
       <c r="G13">
-        <v>22.01619998931885</v>
+        <v>22.10839996337891</v>
       </c>
       <c r="H13">
-        <v>19.22960001627604</v>
+        <v>19.29646667480469</v>
       </c>
       <c r="I13">
-        <v>17.65579999923706</v>
+        <v>17.73019999504089</v>
       </c>
       <c r="J13">
-        <v>16.52159999370575</v>
+        <v>16.5700999879837</v>
       </c>
       <c r="K13">
         <v>10.17000007629395</v>
       </c>
       <c r="L13">
-        <v>24.84000015258789</v>
+        <v>25.8799991607666</v>
       </c>
       <c r="M13">
-        <v>23.52063350908888</v>
+        <v>23.88702688804694</v>
       </c>
       <c r="N13">
-        <v>96.05367011058257</v>
+        <v>100.1546678263189</v>
       </c>
       <c r="O13">
-        <v>164.8632211045166</v>
+        <v>169.0007698888454</v>
       </c>
       <c r="P13">
         <v>75</v>
@@ -1536,58 +1548,58 @@
         <v>31</v>
       </c>
       <c r="B14" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="C14" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D14" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="E14">
-        <v>172.6799926757812</v>
+        <v>19.79000091552734</v>
       </c>
       <c r="F14">
-        <v>573276.6666666666</v>
+        <v>1427620</v>
       </c>
       <c r="G14">
-        <v>150.0152001953125</v>
+        <v>17.07800003051758</v>
       </c>
       <c r="H14">
-        <v>130.9760003153483</v>
+        <v>14.73526666005452</v>
       </c>
       <c r="I14">
-        <v>127.7129001617432</v>
+        <v>13.78679998397827</v>
       </c>
       <c r="J14">
-        <v>120.6059502029419</v>
+        <v>12.8920499753952</v>
       </c>
       <c r="K14">
-        <v>77.62999725341797</v>
+        <v>9</v>
       </c>
       <c r="L14">
-        <v>172.6799926757812</v>
+        <v>19.79000091552734</v>
       </c>
       <c r="M14">
-        <v>26.90525713306577</v>
+        <v>23.6875057220459</v>
       </c>
       <c r="N14">
-        <v>113.5542806979339</v>
+        <v>111.6577551670276</v>
       </c>
       <c r="O14">
-        <v>153.5735734716648</v>
+        <v>166.9688990286866</v>
       </c>
       <c r="P14">
-        <v>35</v>
+        <v>657</v>
       </c>
       <c r="Q14">
-        <v>93</v>
+        <v>139</v>
       </c>
       <c r="R14">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="S14">
-        <v>48.973</v>
+        <v>12.126</v>
       </c>
     </row>
     <row r="15" spans="1:19">
@@ -1595,58 +1607,58 @@
         <v>32</v>
       </c>
       <c r="B15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C15" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D15" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="E15">
-        <v>116.9100036621094</v>
+        <v>315.5199890136719</v>
       </c>
       <c r="F15">
-        <v>833890</v>
+        <v>1841113.333333333</v>
       </c>
       <c r="G15">
-        <v>100.3576007080078</v>
+        <v>273.8059985351563</v>
       </c>
       <c r="H15">
-        <v>94.91413365681966</v>
+        <v>239.3051329549154</v>
       </c>
       <c r="I15">
-        <v>89.35590011596679</v>
+        <v>230.3853998565674</v>
       </c>
       <c r="J15">
-        <v>84.4131000328064</v>
+        <v>218.1875501251221</v>
       </c>
       <c r="K15">
-        <v>53.47000122070312</v>
+        <v>156.25</v>
       </c>
       <c r="L15">
-        <v>116.9100036621094</v>
+        <v>315.5199890136719</v>
       </c>
       <c r="M15">
-        <v>27.82637746817713</v>
+        <v>32.48792655893058</v>
       </c>
       <c r="N15">
-        <v>115.3038771726475</v>
+        <v>92.81348703893424</v>
       </c>
       <c r="O15">
-        <v>151.8327981091966</v>
+        <v>153.8047035305713</v>
       </c>
       <c r="P15">
-        <v>382</v>
+        <v>31</v>
       </c>
       <c r="Q15">
-        <v>1472</v>
+        <v>31</v>
       </c>
       <c r="R15">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="S15">
-        <v>60.964</v>
+        <v>17.834</v>
       </c>
     </row>
     <row r="16" spans="1:19">
@@ -1654,58 +1666,58 @@
         <v>33</v>
       </c>
       <c r="B16" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C16" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="D16" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="E16">
-        <v>309.8099975585938</v>
+        <v>53.95999908447266</v>
       </c>
       <c r="F16">
-        <v>1814770</v>
+        <v>361926.6666666667</v>
       </c>
       <c r="G16">
-        <v>272.2851986694336</v>
+        <v>47.15500015258789</v>
       </c>
       <c r="H16">
-        <v>238.6422663370768</v>
+        <v>41.81273338317871</v>
       </c>
       <c r="I16">
-        <v>229.7257498931885</v>
+        <v>39.25420003890991</v>
       </c>
       <c r="J16">
-        <v>217.6199002075195</v>
+        <v>37.10135003089905</v>
       </c>
       <c r="K16">
-        <v>156.25</v>
+        <v>24.36000061035156</v>
       </c>
       <c r="L16">
-        <v>309.8099975585938</v>
+        <v>53.95999908447266</v>
       </c>
       <c r="M16">
-        <v>30.6498507903709</v>
+        <v>21.55890927328084</v>
       </c>
       <c r="N16">
-        <v>88.28856825090443</v>
+        <v>101.7196227456921</v>
       </c>
       <c r="O16">
-        <v>151.5166803317298</v>
+        <v>150.5488968869894</v>
       </c>
       <c r="P16">
-        <v>31</v>
+        <v>375</v>
       </c>
       <c r="Q16">
-        <v>31</v>
+        <v>129</v>
       </c>
       <c r="R16">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="S16">
-        <v>17.834</v>
+        <v>11.623</v>
       </c>
     </row>
     <row r="17" spans="1:19">
@@ -1713,58 +1725,58 @@
         <v>34</v>
       </c>
       <c r="B17" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C17" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="D17" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="E17">
-        <v>53.02999877929688</v>
+        <v>172.5599975585938</v>
       </c>
       <c r="F17">
-        <v>366686.6666666667</v>
+        <v>561016.6666666666</v>
       </c>
       <c r="G17">
-        <v>46.89560020446778</v>
+        <v>150.8682000732422</v>
       </c>
       <c r="H17">
-        <v>41.67866671244303</v>
+        <v>131.2675336201986</v>
       </c>
       <c r="I17">
-        <v>39.13110004425049</v>
+        <v>128.0637501525879</v>
       </c>
       <c r="J17">
-        <v>37.00805003166199</v>
+        <v>120.9882002258301</v>
       </c>
       <c r="K17">
-        <v>24.36000061035156</v>
+        <v>77.62999725341797</v>
       </c>
       <c r="L17">
-        <v>53.02999877929688</v>
+        <v>172.6799926757812</v>
       </c>
       <c r="M17">
-        <v>22.95385454673782</v>
+        <v>23.99223958393293</v>
       </c>
       <c r="N17">
-        <v>99.43587241437339</v>
+        <v>116.4575952286617</v>
       </c>
       <c r="O17">
-        <v>150.8113817554991</v>
+        <v>150.3446176686472</v>
       </c>
       <c r="P17">
-        <v>375</v>
+        <v>35</v>
       </c>
       <c r="Q17">
-        <v>129</v>
+        <v>93</v>
       </c>
       <c r="R17">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="S17">
-        <v>11.623</v>
+        <v>48.973</v>
       </c>
     </row>
     <row r="18" spans="1:19">
@@ -1772,31 +1784,31 @@
         <v>35</v>
       </c>
       <c r="B18" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C18" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D18" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="E18">
-        <v>47.88000106811523</v>
+        <v>48.90000152587891</v>
       </c>
       <c r="F18">
-        <v>253296.6666666667</v>
+        <v>255593.3333333333</v>
       </c>
       <c r="G18">
-        <v>44.06859970092773</v>
+        <v>44.29939971923828</v>
       </c>
       <c r="H18">
-        <v>36.6288665898641</v>
+        <v>36.75359992980957</v>
       </c>
       <c r="I18">
-        <v>35.05529991149902</v>
+        <v>35.15249992370605</v>
       </c>
       <c r="J18">
-        <v>33.22924993515014</v>
+        <v>33.33149993896485</v>
       </c>
       <c r="K18">
         <v>27.70000076293945</v>
@@ -1805,13 +1817,13 @@
         <v>50.77000045776367</v>
       </c>
       <c r="M18">
-        <v>27.91878353656983</v>
+        <v>29.63944841825585</v>
       </c>
       <c r="N18">
-        <v>61.86612978907806</v>
+        <v>60.38045881587617</v>
       </c>
       <c r="O18">
-        <v>147.664210102652</v>
+        <v>150.1439564494002</v>
       </c>
       <c r="P18">
         <v>1433</v>
@@ -1834,55 +1846,55 @@
         <v>64</v>
       </c>
       <c r="C19" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D19" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="E19">
-        <v>138.7799987792969</v>
+        <v>116.3399963378906</v>
       </c>
       <c r="F19">
-        <v>1080943.333333333</v>
+        <v>779956.6666666666</v>
       </c>
       <c r="G19">
-        <v>119.3484004211426</v>
+        <v>100.851400604248</v>
       </c>
       <c r="H19">
-        <v>103.4166668192546</v>
+        <v>95.12473363240559</v>
       </c>
       <c r="I19">
-        <v>103.0755001068115</v>
+        <v>89.62155010223388</v>
       </c>
       <c r="J19">
-        <v>99.47989997863769</v>
+        <v>84.64790002822876</v>
       </c>
       <c r="K19">
-        <v>73.19999694824219</v>
+        <v>53.47000122070312</v>
       </c>
       <c r="L19">
-        <v>139.2100067138672</v>
+        <v>116.9100036621094</v>
       </c>
       <c r="M19">
-        <v>29.78583969252961</v>
+        <v>21.50391262442886</v>
       </c>
       <c r="N19">
-        <v>84.44976438007568</v>
+        <v>117.5799395584169</v>
       </c>
       <c r="O19">
-        <v>146.1299774179572</v>
+        <v>149.4281120511799</v>
       </c>
       <c r="P19">
-        <v>789</v>
+        <v>382</v>
       </c>
       <c r="Q19">
-        <v>27</v>
+        <v>1472</v>
       </c>
       <c r="R19">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="S19">
-        <v>38.525</v>
+        <v>60.964</v>
       </c>
     </row>
     <row r="20" spans="1:19">
@@ -1890,58 +1902,58 @@
         <v>37</v>
       </c>
       <c r="B20" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C20" t="s">
-        <v>68</v>
+        <v>83</v>
       </c>
       <c r="D20" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="E20">
-        <v>77.65000152587891</v>
+        <v>124.4199981689453</v>
       </c>
       <c r="F20">
-        <v>820823.3333333334</v>
+        <v>2314573.333333333</v>
       </c>
       <c r="G20">
-        <v>67.0271996307373</v>
+        <v>107.3230001831055</v>
       </c>
       <c r="H20">
-        <v>60.32859990437826</v>
+        <v>94.73746688842773</v>
       </c>
       <c r="I20">
-        <v>59.40624988555908</v>
+        <v>91.84310009002685</v>
       </c>
       <c r="J20">
-        <v>56.70214996337891</v>
+        <v>87.48230010986327</v>
       </c>
       <c r="K20">
-        <v>42.77000045776367</v>
+        <v>68.48000335693359</v>
       </c>
       <c r="L20">
-        <v>77.65000152587891</v>
+        <v>124.4199981689453</v>
       </c>
       <c r="M20">
-        <v>34.27286714035842</v>
+        <v>28.58618791034311</v>
       </c>
       <c r="N20">
-        <v>81.55249168762579</v>
+        <v>77.99713226455596</v>
       </c>
       <c r="O20">
-        <v>145.5842309361661</v>
+        <v>146.0816190800205</v>
       </c>
       <c r="P20">
-        <v>26</v>
+        <v>53</v>
       </c>
       <c r="Q20">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="R20">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="S20">
-        <v>63.88200000000001</v>
+        <v>31.68</v>
       </c>
     </row>
     <row r="21" spans="1:19">
@@ -1949,31 +1961,31 @@
         <v>38</v>
       </c>
       <c r="B21" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C21" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D21" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E21">
-        <v>970.9199829101562</v>
+        <v>990.7899780273438</v>
       </c>
       <c r="F21">
-        <v>1153396.666666667</v>
+        <v>1140813.333333333</v>
       </c>
       <c r="G21">
-        <v>893.9568029785156</v>
+        <v>899.4536022949219</v>
       </c>
       <c r="H21">
-        <v>732.9624015299479</v>
+        <v>735.2580680338542</v>
       </c>
       <c r="I21">
-        <v>726.88955078125</v>
+        <v>728.2325006103515</v>
       </c>
       <c r="J21">
-        <v>698.4728506469727</v>
+        <v>699.9805004882812</v>
       </c>
       <c r="K21">
         <v>570.5999755859375</v>
@@ -1982,13 +1994,13 @@
         <v>1047.390014648438</v>
       </c>
       <c r="M21">
-        <v>30.8411700003397</v>
+        <v>33.04195093518072</v>
       </c>
       <c r="N21">
-        <v>46.18766896072333</v>
+        <v>53.01066100412362</v>
       </c>
       <c r="O21">
-        <v>144.8893435855737</v>
+        <v>145.2968196750034</v>
       </c>
       <c r="P21">
         <v>320</v>
@@ -2008,58 +2020,58 @@
         <v>39</v>
       </c>
       <c r="B22" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C22" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="D22" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E22">
-        <v>121.4499969482422</v>
+        <v>78.47000122070312</v>
       </c>
       <c r="F22">
-        <v>2310256.666666667</v>
+        <v>819616.6666666666</v>
       </c>
       <c r="G22">
-        <v>106.731000213623</v>
+        <v>67.45319969177245</v>
       </c>
       <c r="H22">
-        <v>94.47173355102539</v>
+        <v>60.46073323567708</v>
       </c>
       <c r="I22">
-        <v>91.5876501083374</v>
+        <v>59.54839988708496</v>
       </c>
       <c r="J22">
-        <v>87.2935001373291</v>
+        <v>56.83289995193481</v>
       </c>
       <c r="K22">
-        <v>68.48000335693359</v>
+        <v>43.04000091552734</v>
       </c>
       <c r="L22">
-        <v>121.4499969482422</v>
+        <v>78.47000122070312</v>
       </c>
       <c r="M22">
-        <v>26.84072788328167</v>
+        <v>32.75249604203383</v>
       </c>
       <c r="N22">
-        <v>73.97221199772331</v>
+        <v>82.31877219220472</v>
       </c>
       <c r="O22">
-        <v>144.1624755239744</v>
+        <v>145.1858831487718</v>
       </c>
       <c r="P22">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="Q22">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="R22">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="S22">
-        <v>31.68</v>
+        <v>63.88200000000001</v>
       </c>
     </row>
     <row r="23" spans="1:19">
@@ -2067,58 +2079,58 @@
         <v>40</v>
       </c>
       <c r="B23" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="C23" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D23" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E23">
-        <v>67.52999877929688</v>
+        <v>136.2400054931641</v>
       </c>
       <c r="F23">
-        <v>3708030</v>
+        <v>1080700</v>
       </c>
       <c r="G23">
-        <v>61.3147998046875</v>
+        <v>119.904200592041</v>
       </c>
       <c r="H23">
-        <v>53.12666653951009</v>
+        <v>103.6296668497721</v>
       </c>
       <c r="I23">
-        <v>51.98269992828369</v>
+        <v>103.2609001159668</v>
       </c>
       <c r="J23">
-        <v>49.71974994659424</v>
+        <v>99.6518999862671</v>
       </c>
       <c r="K23">
-        <v>40.18999862670898</v>
+        <v>73.19999694824219</v>
       </c>
       <c r="L23">
-        <v>69.37999725341797</v>
+        <v>139.2100067138672</v>
       </c>
       <c r="M23">
-        <v>26.95995586167803</v>
+        <v>28.00902480739595</v>
       </c>
       <c r="N23">
-        <v>68.02687506045</v>
+        <v>78.9805577736682</v>
       </c>
       <c r="O23">
-        <v>142.7943920177864</v>
+        <v>143.2884880758006</v>
       </c>
       <c r="P23">
-        <v>492</v>
+        <v>789</v>
       </c>
       <c r="Q23">
-        <v>65</v>
+        <v>27</v>
       </c>
       <c r="R23">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="S23">
-        <v>20.031</v>
+        <v>38.525</v>
       </c>
     </row>
     <row r="24" spans="1:19">
@@ -2126,46 +2138,46 @@
         <v>41</v>
       </c>
       <c r="B24" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C24" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D24" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E24">
-        <v>603.6400146484375</v>
+        <v>612.9500122070312</v>
       </c>
       <c r="F24">
-        <v>508540</v>
+        <v>506823.3333333333</v>
       </c>
       <c r="G24">
-        <v>543.7805999755859</v>
+        <v>546.0932000732422</v>
       </c>
       <c r="H24">
-        <v>478.8650004069011</v>
+        <v>479.9378672281901</v>
       </c>
       <c r="I24">
-        <v>470.7074011230468</v>
+        <v>471.6868011474609</v>
       </c>
       <c r="J24">
-        <v>452.0413012695312</v>
+        <v>452.7938011169434</v>
       </c>
       <c r="K24">
-        <v>333.4500122070312</v>
+        <v>336.8299865722656</v>
       </c>
       <c r="L24">
-        <v>611.9099731445312</v>
+        <v>612.9500122070312</v>
       </c>
       <c r="M24">
-        <v>23.09386337753825</v>
+        <v>24.36847004487821</v>
       </c>
       <c r="N24">
-        <v>81.02863774185489</v>
+        <v>81.97608189362472</v>
       </c>
       <c r="O24">
-        <v>142.057408377519</v>
+        <v>142.2097810266116</v>
       </c>
       <c r="P24">
         <v>54</v>
@@ -2185,58 +2197,58 @@
         <v>42</v>
       </c>
       <c r="B25" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C25" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="D25" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="E25">
-        <v>546.4600219726562</v>
+        <v>194.8099975585938</v>
       </c>
       <c r="F25">
-        <v>579576.6666666666</v>
+        <v>650253.3333333334</v>
       </c>
       <c r="G25">
-        <v>507.783998413086</v>
+        <v>179.0701998901367</v>
       </c>
       <c r="H25">
-        <v>444.6837986246745</v>
+        <v>154.4811334228516</v>
       </c>
       <c r="I25">
-        <v>431.0207997131347</v>
+        <v>149.8068500518799</v>
       </c>
       <c r="J25">
-        <v>410.4548500061035</v>
+        <v>144.0530000305176</v>
       </c>
       <c r="K25">
-        <v>311.6499938964844</v>
+        <v>123.25</v>
       </c>
       <c r="L25">
-        <v>546.4600219726562</v>
+        <v>195.5700073242188</v>
       </c>
       <c r="M25">
-        <v>20.50101076988093</v>
+        <v>25.61903227910793</v>
       </c>
       <c r="N25">
-        <v>70.54490951636565</v>
+        <v>58.00956777676449</v>
       </c>
       <c r="O25">
-        <v>139.6274422488626</v>
+        <v>141.581383444262</v>
       </c>
       <c r="P25">
-        <v>72</v>
+        <v>115</v>
       </c>
       <c r="Q25">
-        <v>59</v>
+        <v>166</v>
       </c>
       <c r="R25">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S25">
-        <v>25.507</v>
+        <v>8.3500005</v>
       </c>
     </row>
     <row r="26" spans="1:19">
@@ -2244,58 +2256,58 @@
         <v>43</v>
       </c>
       <c r="B26" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C26" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="D26" t="s">
-        <v>116</v>
+        <v>101</v>
       </c>
       <c r="E26">
-        <v>178.1499938964844</v>
+        <v>560.6400146484375</v>
       </c>
       <c r="F26">
-        <v>42134630</v>
+        <v>582590</v>
       </c>
       <c r="G26">
-        <v>167.397798461914</v>
+        <v>509.8475988769531</v>
       </c>
       <c r="H26">
-        <v>148.4011331176758</v>
+        <v>445.7125986735026</v>
       </c>
       <c r="I26">
-        <v>143.9355000305176</v>
+        <v>432.1370997619629</v>
       </c>
       <c r="J26">
-        <v>137.8724501800537</v>
+        <v>411.4383500671387</v>
       </c>
       <c r="K26">
-        <v>97.23999786376953</v>
+        <v>311.6499938964844</v>
       </c>
       <c r="L26">
-        <v>178.75</v>
+        <v>560.6400146484375</v>
       </c>
       <c r="M26">
-        <v>15.62924996919917</v>
+        <v>21.80941266957526</v>
       </c>
       <c r="N26">
-        <v>80.47816386263935</v>
+        <v>74.72497372142313</v>
       </c>
       <c r="O26">
-        <v>138.7637963501963</v>
+        <v>141.5347281644603</v>
       </c>
       <c r="P26">
-        <v>3233</v>
+        <v>72</v>
       </c>
       <c r="Q26">
-        <v>1174</v>
+        <v>59</v>
       </c>
       <c r="R26">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="S26">
-        <v>17.49</v>
+        <v>25.507</v>
       </c>
     </row>
     <row r="27" spans="1:19">
@@ -2303,58 +2315,58 @@
         <v>44</v>
       </c>
       <c r="B27" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C27" t="s">
-        <v>74</v>
+        <v>87</v>
       </c>
       <c r="D27" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E27">
-        <v>190.3800048828125</v>
+        <v>67.68000030517578</v>
       </c>
       <c r="F27">
-        <v>650326.6666666666</v>
+        <v>3732893.333333333</v>
       </c>
       <c r="G27">
-        <v>178.2169998168945</v>
+        <v>61.59419982910156</v>
       </c>
       <c r="H27">
-        <v>154.0985334269206</v>
+        <v>53.25219988505046</v>
       </c>
       <c r="I27">
-        <v>149.4903000640869</v>
+        <v>52.09709993362426</v>
       </c>
       <c r="J27">
-        <v>143.8183499908447</v>
+        <v>49.82504993438721</v>
       </c>
       <c r="K27">
-        <v>123.25</v>
+        <v>40.25</v>
       </c>
       <c r="L27">
-        <v>195.5700073242188</v>
+        <v>69.37999725341797</v>
       </c>
       <c r="M27">
-        <v>22.90510805961588</v>
+        <v>26.15097554569368</v>
       </c>
       <c r="N27">
-        <v>53.85486356029334</v>
+        <v>68.14906908118206</v>
       </c>
       <c r="O27">
-        <v>138.7342883590967</v>
+        <v>140.9253429133988</v>
       </c>
       <c r="P27">
-        <v>115</v>
+        <v>492</v>
       </c>
       <c r="Q27">
-        <v>166</v>
+        <v>65</v>
       </c>
       <c r="R27">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="S27">
-        <v>8.3500005</v>
+        <v>20.031</v>
       </c>
     </row>
     <row r="28" spans="1:19">
@@ -2362,58 +2374,58 @@
         <v>45</v>
       </c>
       <c r="B28" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C28" t="s">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="D28" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="E28">
-        <v>101.120002746582</v>
+        <v>415</v>
       </c>
       <c r="F28">
-        <v>1832483.333333333</v>
+        <v>420759.5</v>
       </c>
       <c r="G28">
-        <v>91.49139938354492</v>
+        <v>361.4619995117188</v>
       </c>
       <c r="H28">
-        <v>80.25359985351562</v>
+        <v>325.1172668457031</v>
       </c>
       <c r="I28">
-        <v>78.2484497833252</v>
+        <v>323.5828999328613</v>
       </c>
       <c r="J28">
-        <v>75.51434986114502</v>
+        <v>312.6676502990722</v>
       </c>
       <c r="K28">
-        <v>65.79000091552734</v>
+        <v>221.2799987792969</v>
       </c>
       <c r="L28">
-        <v>101.120002746582</v>
+        <v>415</v>
       </c>
       <c r="M28">
-        <v>25.67736005119641</v>
+        <v>28.20908797611768</v>
       </c>
       <c r="N28">
-        <v>53.70117242651735</v>
+        <v>80.2153909153617</v>
       </c>
       <c r="O28">
-        <v>137.6277629066684</v>
+        <v>138.424202572195</v>
       </c>
       <c r="P28">
-        <v>39</v>
+        <v>465</v>
       </c>
       <c r="Q28">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="R28">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="S28">
-        <v>17.267</v>
+        <v>29.126</v>
       </c>
     </row>
     <row r="29" spans="1:19">
@@ -2421,58 +2433,58 @@
         <v>46</v>
       </c>
       <c r="B29" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C29" t="s">
-        <v>67</v>
+        <v>88</v>
       </c>
       <c r="D29" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="E29">
-        <v>406.6499938964844</v>
+        <v>178.1499938964844</v>
       </c>
       <c r="F29">
-        <v>424360.4666666667</v>
+        <v>41657526.66666666</v>
       </c>
       <c r="G29">
-        <v>359.7169995117188</v>
+        <v>167.9333984375</v>
       </c>
       <c r="H29">
-        <v>324.3940667724609</v>
+        <v>148.6883330281576</v>
       </c>
       <c r="I29">
-        <v>322.9790998840332</v>
+        <v>144.1997499847412</v>
       </c>
       <c r="J29">
-        <v>312.2045002746582</v>
+        <v>138.2170501708984</v>
       </c>
       <c r="K29">
-        <v>221.2799987792969</v>
+        <v>97.23999786376953</v>
       </c>
       <c r="L29">
-        <v>406.6499938964844</v>
+        <v>178.75</v>
       </c>
       <c r="M29">
-        <v>25.08074566111753</v>
+        <v>15.83978260863095</v>
       </c>
       <c r="N29">
-        <v>75.55257941977736</v>
+        <v>81.54488829385882</v>
       </c>
       <c r="O29">
-        <v>137.5260737277241</v>
+        <v>137.6863502325201</v>
       </c>
       <c r="P29">
-        <v>465</v>
+        <v>3233</v>
       </c>
       <c r="Q29">
-        <v>40</v>
+        <v>1174</v>
       </c>
       <c r="R29">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="S29">
-        <v>29.126</v>
+        <v>17.49</v>
       </c>
     </row>
     <row r="30" spans="1:19">
@@ -2480,31 +2492,31 @@
         <v>47</v>
       </c>
       <c r="B30" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C30" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D30" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E30">
-        <v>104.4400024414062</v>
+        <v>105.0699996948242</v>
       </c>
       <c r="F30">
-        <v>2440580</v>
+        <v>2447396.666666667</v>
       </c>
       <c r="G30">
-        <v>91.91079956054688</v>
+        <v>92.29079956054687</v>
       </c>
       <c r="H30">
-        <v>83.6765995279948</v>
+        <v>83.87433283487955</v>
       </c>
       <c r="I30">
-        <v>81.75914978027343</v>
+        <v>81.93309978485108</v>
       </c>
       <c r="J30">
-        <v>78.52464977264404</v>
+        <v>78.63554977416992</v>
       </c>
       <c r="K30">
         <v>60.77999877929688</v>
@@ -2513,13 +2525,13 @@
         <v>105.3099975585938</v>
       </c>
       <c r="M30">
-        <v>16.43255963728649</v>
+        <v>15.93291722279255</v>
       </c>
       <c r="N30">
-        <v>69.73834635691134</v>
+        <v>72.07664155209821</v>
       </c>
       <c r="O30">
-        <v>136.6520641234111</v>
+        <v>137.3618764862367</v>
       </c>
       <c r="P30">
         <v>393</v>
@@ -2539,58 +2551,58 @@
         <v>48</v>
       </c>
       <c r="B31" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="C31" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="D31" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="E31">
-        <v>767.5599975585938</v>
+        <v>100.5500030517578</v>
       </c>
       <c r="F31">
-        <v>1251926.666666667</v>
+        <v>1825316.666666667</v>
       </c>
       <c r="G31">
-        <v>763.6093994140625</v>
+        <v>91.86499938964843</v>
       </c>
       <c r="H31">
-        <v>663.8521988932291</v>
+        <v>80.4416665649414</v>
       </c>
       <c r="I31">
-        <v>638.4068994140625</v>
+        <v>78.40149978637696</v>
       </c>
       <c r="J31">
-        <v>611.3496002197265</v>
+        <v>75.63829982757568</v>
       </c>
       <c r="K31">
-        <v>429.0799865722656</v>
+        <v>66.12000274658203</v>
       </c>
       <c r="L31">
-        <v>812.9400024414062</v>
+        <v>101.120002746582</v>
       </c>
       <c r="M31">
-        <v>9.071794110330945</v>
+        <v>24.07453345979953</v>
       </c>
       <c r="N31">
-        <v>74.25931287747289</v>
+        <v>52.0719886191408</v>
       </c>
       <c r="O31">
-        <v>136.0852233020913</v>
+        <v>136.6212372755077</v>
       </c>
       <c r="P31">
-        <v>93</v>
+        <v>39</v>
       </c>
       <c r="Q31">
-        <v>426</v>
+        <v>46</v>
       </c>
       <c r="R31">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="S31">
-        <v>27.346</v>
+        <v>17.267</v>
       </c>
     </row>
     <row r="32" spans="1:19">
@@ -2598,58 +2610,58 @@
         <v>49</v>
       </c>
       <c r="B32" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C32" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D32" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="E32">
-        <v>81.33000183105469</v>
+        <v>773.1799926757812</v>
       </c>
       <c r="F32">
-        <v>10707240</v>
+        <v>1263653.333333333</v>
       </c>
       <c r="G32">
-        <v>79.53420013427734</v>
+        <v>765.099599609375</v>
       </c>
       <c r="H32">
-        <v>68.25639999389648</v>
+        <v>665.343398844401</v>
       </c>
       <c r="I32">
-        <v>66.96285001754761</v>
+        <v>639.4892492675781</v>
       </c>
       <c r="J32">
-        <v>65.35520002365112</v>
+        <v>613.021650390625</v>
       </c>
       <c r="K32">
-        <v>44.31000137329102</v>
+        <v>429.0799865722656</v>
       </c>
       <c r="L32">
-        <v>90.72000122070312</v>
+        <v>812.9400024414062</v>
       </c>
       <c r="M32">
-        <v>5.445358131982303</v>
+        <v>9.250959951172577</v>
       </c>
       <c r="N32">
-        <v>77.61520027285206</v>
+        <v>78.60475943103502</v>
       </c>
       <c r="O32">
-        <v>135.5862827541882</v>
+        <v>136.4504177976586</v>
       </c>
       <c r="P32">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="Q32">
-        <v>104</v>
+        <v>426</v>
       </c>
       <c r="R32">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="S32">
-        <v>1.526</v>
+        <v>27.346</v>
       </c>
     </row>
     <row r="33" spans="1:19">
@@ -2657,58 +2669,58 @@
         <v>50</v>
       </c>
       <c r="B33" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="C33" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D33" t="s">
-        <v>123</v>
+        <v>101</v>
       </c>
       <c r="E33">
-        <v>146.6799926757812</v>
+        <v>199.0599975585938</v>
       </c>
       <c r="F33">
-        <v>1229720</v>
+        <v>8037060</v>
       </c>
       <c r="G33">
-        <v>130.6763996887207</v>
+        <v>179.8067993164063</v>
       </c>
       <c r="H33">
-        <v>118.6953329467773</v>
+        <v>160.8138663736979</v>
       </c>
       <c r="I33">
-        <v>115.3791497802734</v>
+        <v>157.7651997375488</v>
       </c>
       <c r="J33">
-        <v>111.6238998794556</v>
+        <v>152.5785498809815</v>
       </c>
       <c r="K33">
-        <v>95.08999633789062</v>
+        <v>124.9100036621094</v>
       </c>
       <c r="L33">
-        <v>148.4499969482422</v>
+        <v>199.0599975585938</v>
       </c>
       <c r="M33">
-        <v>15.98924065925547</v>
+        <v>18.17156495393512</v>
       </c>
       <c r="N33">
-        <v>54.25386299792451</v>
+        <v>59.36273454691867</v>
       </c>
       <c r="O33">
-        <v>133.4610122962561</v>
+        <v>134.212745271289</v>
       </c>
       <c r="P33">
-        <v>254</v>
+        <v>369</v>
       </c>
       <c r="Q33">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="R33">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="S33">
-        <v>19.516</v>
+        <v>15.979</v>
       </c>
     </row>
     <row r="34" spans="1:19">
@@ -2716,58 +2728,58 @@
         <v>51</v>
       </c>
       <c r="B34" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C34" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D34" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="E34">
-        <v>196.3300018310547</v>
+        <v>148.1399993896484</v>
       </c>
       <c r="F34">
-        <v>7905863.333333333</v>
+        <v>1227063.333333333</v>
       </c>
       <c r="G34">
-        <v>179.2387994384766</v>
+        <v>131.2015997314453</v>
       </c>
       <c r="H34">
-        <v>160.48806640625</v>
+        <v>119.0007996114095</v>
       </c>
       <c r="I34">
-        <v>157.4653497314453</v>
+        <v>115.5921997833252</v>
       </c>
       <c r="J34">
-        <v>152.3468998718262</v>
+        <v>111.7746998977661</v>
       </c>
       <c r="K34">
-        <v>124.9100036621094</v>
+        <v>95.19999694824219</v>
       </c>
       <c r="L34">
-        <v>196.3300018310547</v>
+        <v>148.4499969482422</v>
       </c>
       <c r="M34">
-        <v>18.10744563385018</v>
+        <v>16.60894074469592</v>
       </c>
       <c r="N34">
-        <v>54.78556251929303</v>
+        <v>54.4412033127099</v>
       </c>
       <c r="O34">
-        <v>132.8664916076386</v>
+        <v>133.8670389992105</v>
       </c>
       <c r="P34">
-        <v>369</v>
+        <v>254</v>
       </c>
       <c r="Q34">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="R34">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="S34">
-        <v>15.979</v>
+        <v>19.516</v>
       </c>
     </row>
     <row r="35" spans="1:19">
@@ -2775,46 +2787,46 @@
         <v>52</v>
       </c>
       <c r="B35" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C35" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D35" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="E35">
-        <v>251.1399993896484</v>
+        <v>252.9199981689453</v>
       </c>
       <c r="F35">
-        <v>373796.6666666667</v>
+        <v>368583.3333333333</v>
       </c>
       <c r="G35">
-        <v>240.1861996459961</v>
+        <v>241.1643997192383</v>
       </c>
       <c r="H35">
-        <v>217.6723329671224</v>
+        <v>218.0927329508463</v>
       </c>
       <c r="I35">
-        <v>211.2792997741699</v>
+        <v>211.6189497375488</v>
       </c>
       <c r="J35">
-        <v>203.5096997833252</v>
+        <v>203.9065497589111</v>
       </c>
       <c r="K35">
-        <v>146.3999938964844</v>
+        <v>147.3000030517578</v>
       </c>
       <c r="L35">
         <v>266.0299987792969</v>
       </c>
       <c r="M35">
-        <v>14.91718088452243</v>
+        <v>13.96386541517962</v>
       </c>
       <c r="N35">
-        <v>71.54372258186226</v>
+        <v>71.70400063065516</v>
       </c>
       <c r="O35">
-        <v>132.7688763338003</v>
+        <v>132.4779964810827</v>
       </c>
       <c r="P35">
         <v>342</v>
@@ -2834,58 +2846,58 @@
         <v>53</v>
       </c>
       <c r="B36" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C36" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="D36" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E36">
-        <v>416.1000061035156</v>
+        <v>79.58999633789062</v>
       </c>
       <c r="F36">
-        <v>399356.6666666667</v>
+        <v>10641293.33333333</v>
       </c>
       <c r="G36">
-        <v>385.2098004150391</v>
+        <v>79.52380004882812</v>
       </c>
       <c r="H36">
-        <v>357.9802673339844</v>
+        <v>68.41806663513184</v>
       </c>
       <c r="I36">
-        <v>343.2438005065918</v>
+        <v>67.06120000839233</v>
       </c>
       <c r="J36">
-        <v>331.8901504516601</v>
+        <v>65.42020002365112</v>
       </c>
       <c r="K36">
-        <v>263.6799926757812</v>
+        <v>44.31000137329102</v>
       </c>
       <c r="L36">
-        <v>419.5299987792969</v>
+        <v>90.72000122070312</v>
       </c>
       <c r="M36">
-        <v>13.61402828708922</v>
+        <v>1.582639295365262</v>
       </c>
       <c r="N36">
-        <v>57.80492174662215</v>
+        <v>76.94530268537558</v>
       </c>
       <c r="O36">
-        <v>131.7686969390251</v>
+        <v>132.3953036225388</v>
       </c>
       <c r="P36">
-        <v>339</v>
+        <v>84</v>
       </c>
       <c r="Q36">
-        <v>39</v>
+        <v>104</v>
       </c>
       <c r="R36">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="S36">
-        <v>30.394</v>
+        <v>1.526</v>
       </c>
     </row>
     <row r="37" spans="1:19">
@@ -2893,58 +2905,58 @@
         <v>54</v>
       </c>
       <c r="B37" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C37" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D37" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E37">
-        <v>86.69999694824219</v>
+        <v>417.75</v>
       </c>
       <c r="F37">
-        <v>1160050</v>
+        <v>390360</v>
       </c>
       <c r="G37">
-        <v>80.64440032958984</v>
+        <v>385.9556005859375</v>
       </c>
       <c r="H37">
-        <v>74.74946665445964</v>
+        <v>358.6686006673177</v>
       </c>
       <c r="I37">
-        <v>73.13319997787475</v>
+        <v>343.8668504333496</v>
       </c>
       <c r="J37">
-        <v>71.11359996795655</v>
+        <v>332.4139004516601</v>
       </c>
       <c r="K37">
-        <v>55.06000137329102</v>
+        <v>265.4599914550781</v>
       </c>
       <c r="L37">
-        <v>86.69999694824219</v>
+        <v>419.5299987792969</v>
       </c>
       <c r="M37">
-        <v>22.0610987445387</v>
+        <v>16.2839248434238</v>
       </c>
       <c r="N37">
-        <v>57.46457462004238</v>
+        <v>56.03989171343797</v>
       </c>
       <c r="O37">
-        <v>131.4849912865098</v>
+        <v>131.2903748443835</v>
       </c>
       <c r="P37">
-        <v>84</v>
+        <v>339</v>
       </c>
       <c r="Q37">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="R37">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="S37">
-        <v>17.093</v>
+        <v>30.394</v>
       </c>
     </row>
     <row r="38" spans="1:19">
@@ -2952,46 +2964,46 @@
         <v>55</v>
       </c>
       <c r="B38" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C38" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D38" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="E38">
-        <v>589.780029296875</v>
+        <v>602.010009765625</v>
       </c>
       <c r="F38">
-        <v>1088726.666666667</v>
+        <v>1114300</v>
       </c>
       <c r="G38">
-        <v>551.9458013916015</v>
+        <v>553.9486016845703</v>
       </c>
       <c r="H38">
-        <v>511.3422025553385</v>
+        <v>512.5008693440756</v>
       </c>
       <c r="I38">
-        <v>493.7417015075683</v>
+        <v>494.5009515380859</v>
       </c>
       <c r="J38">
-        <v>476.6125509643555</v>
+        <v>477.6592510986328</v>
       </c>
       <c r="K38">
         <v>364.5299987792969</v>
       </c>
       <c r="L38">
-        <v>594.3200073242188</v>
+        <v>602.010009765625</v>
       </c>
       <c r="M38">
-        <v>5.376195165933639</v>
+        <v>7.761565104564427</v>
       </c>
       <c r="N38">
-        <v>55.45072187265001</v>
+        <v>59.87094053237841</v>
       </c>
       <c r="O38">
-        <v>128.9749612378913</v>
+        <v>130.6536797682308</v>
       </c>
       <c r="P38">
         <v>65</v>
@@ -3011,58 +3023,58 @@
         <v>56</v>
       </c>
       <c r="B39" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="C39" t="s">
+        <v>93</v>
+      </c>
+      <c r="D39" t="s">
+        <v>130</v>
+      </c>
+      <c r="E39">
+        <v>86.04000091552734</v>
+      </c>
+      <c r="F39">
+        <v>1165633.333333333</v>
+      </c>
+      <c r="G39">
+        <v>80.92780029296875</v>
+      </c>
+      <c r="H39">
+        <v>74.84086664835613</v>
+      </c>
+      <c r="I39">
+        <v>73.24499998092651</v>
+      </c>
+      <c r="J39">
+        <v>71.20764999389648</v>
+      </c>
+      <c r="K39">
+        <v>55.36000061035156</v>
+      </c>
+      <c r="L39">
+        <v>86.69999694824219</v>
+      </c>
+      <c r="M39">
+        <v>21.30269356455787</v>
+      </c>
+      <c r="N39">
+        <v>55.41907508476262</v>
+      </c>
+      <c r="O39">
+        <v>129.8661207712484</v>
+      </c>
+      <c r="P39">
         <v>84</v>
       </c>
-      <c r="D39" t="s">
-        <v>128</v>
-      </c>
-      <c r="E39">
-        <v>149.1699981689453</v>
-      </c>
-      <c r="F39">
-        <v>305556.6666666667</v>
-      </c>
-      <c r="G39">
-        <v>140.2481991577149</v>
-      </c>
-      <c r="H39">
-        <v>133.2301329549154</v>
-      </c>
-      <c r="I39">
-        <v>129.7500496292114</v>
-      </c>
-      <c r="J39">
-        <v>126.1467496490478</v>
-      </c>
-      <c r="K39">
-        <v>89.83000183105469</v>
-      </c>
-      <c r="L39">
-        <v>149.4199981689453</v>
-      </c>
-      <c r="M39">
-        <v>9.869627660608661</v>
-      </c>
-      <c r="N39">
-        <v>66.05810433967562</v>
-      </c>
-      <c r="O39">
-        <v>126.0097083154118</v>
-      </c>
-      <c r="P39">
-        <v>198</v>
-      </c>
       <c r="Q39">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="R39">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="S39">
-        <v>14.181</v>
+        <v>17.093</v>
       </c>
     </row>
     <row r="40" spans="1:19">
@@ -3070,58 +3082,176 @@
         <v>57</v>
       </c>
       <c r="B40" t="s">
+        <v>64</v>
+      </c>
+      <c r="C40" t="s">
+        <v>94</v>
+      </c>
+      <c r="D40" t="s">
+        <v>131</v>
+      </c>
+      <c r="E40">
+        <v>38.25</v>
+      </c>
+      <c r="F40">
+        <v>787773.3333333334</v>
+      </c>
+      <c r="G40">
+        <v>37.71040016174317</v>
+      </c>
+      <c r="H40">
+        <v>35.63240002950032</v>
+      </c>
+      <c r="I40">
+        <v>33.1810000038147</v>
+      </c>
+      <c r="J40">
+        <v>31.78385003089905</v>
+      </c>
+      <c r="K40">
+        <v>19.52000045776367</v>
+      </c>
+      <c r="L40">
+        <v>47.79999923706055</v>
+      </c>
+      <c r="M40">
+        <v>0</v>
+      </c>
+      <c r="N40">
+        <v>85.1403692279854</v>
+      </c>
+      <c r="O40">
+        <v>128.221449349329</v>
+      </c>
+      <c r="P40">
+        <v>94</v>
+      </c>
+      <c r="Q40">
+        <v>141</v>
+      </c>
+      <c r="R40">
+        <v>58</v>
+      </c>
+      <c r="S40">
+        <v>33.405998</v>
+      </c>
+    </row>
+    <row r="41" spans="1:19">
+      <c r="A41" t="s">
+        <v>58</v>
+      </c>
+      <c r="B41" t="s">
+        <v>61</v>
+      </c>
+      <c r="C41" t="s">
+        <v>95</v>
+      </c>
+      <c r="D41" t="s">
+        <v>132</v>
+      </c>
+      <c r="E41">
+        <v>32.88999938964844</v>
+      </c>
+      <c r="F41">
+        <v>870953.3333333334</v>
+      </c>
+      <c r="G41">
+        <v>30.89800010681152</v>
+      </c>
+      <c r="H41">
+        <v>29.23626664479574</v>
+      </c>
+      <c r="I41">
+        <v>28.82175002098084</v>
+      </c>
+      <c r="J41">
+        <v>27.86904999732971</v>
+      </c>
+      <c r="K41">
+        <v>19.85000038146973</v>
+      </c>
+      <c r="L41">
+        <v>33.25</v>
+      </c>
+      <c r="M41">
+        <v>10.480345595934</v>
+      </c>
+      <c r="N41">
+        <v>65.69268895506796</v>
+      </c>
+      <c r="O41">
+        <v>125.6219221815115</v>
+      </c>
+      <c r="P41">
+        <v>688</v>
+      </c>
+      <c r="Q41">
+        <v>60</v>
+      </c>
+      <c r="R41">
+        <v>5</v>
+      </c>
+      <c r="S41">
+        <v>6.476</v>
+      </c>
+    </row>
+    <row r="42" spans="1:19">
+      <c r="A42" t="s">
         <v>59</v>
       </c>
-      <c r="C40" t="s">
-        <v>92</v>
-      </c>
-      <c r="D40" t="s">
-        <v>129</v>
-      </c>
-      <c r="E40">
-        <v>32.58000183105469</v>
-      </c>
-      <c r="F40">
-        <v>960910</v>
-      </c>
-      <c r="G40">
-        <v>30.8010001373291</v>
-      </c>
-      <c r="H40">
-        <v>29.21053332010905</v>
-      </c>
-      <c r="I40">
-        <v>28.77770002365112</v>
-      </c>
-      <c r="J40">
-        <v>27.81964999198913</v>
-      </c>
-      <c r="K40">
-        <v>19.79000091552734</v>
-      </c>
-      <c r="L40">
-        <v>33.25</v>
-      </c>
-      <c r="M40">
-        <v>9.95613484253559</v>
-      </c>
-      <c r="N40">
-        <v>64.62860193953928</v>
-      </c>
-      <c r="O40">
-        <v>125.2618641387009</v>
-      </c>
-      <c r="P40">
-        <v>688</v>
-      </c>
-      <c r="Q40">
-        <v>60</v>
-      </c>
-      <c r="R40">
-        <v>5</v>
-      </c>
-      <c r="S40">
-        <v>6.476</v>
+      <c r="B42" t="s">
+        <v>61</v>
+      </c>
+      <c r="C42" t="s">
+        <v>87</v>
+      </c>
+      <c r="D42" t="s">
+        <v>133</v>
+      </c>
+      <c r="E42">
+        <v>149.2400054931641</v>
+      </c>
+      <c r="F42">
+        <v>304830</v>
+      </c>
+      <c r="G42">
+        <v>140.5671994018555</v>
+      </c>
+      <c r="H42">
+        <v>133.3882663472494</v>
+      </c>
+      <c r="I42">
+        <v>129.9510996627808</v>
+      </c>
+      <c r="J42">
+        <v>126.2975996780395</v>
+      </c>
+      <c r="K42">
+        <v>90.83000183105469</v>
+      </c>
+      <c r="L42">
+        <v>149.4199981689453</v>
+      </c>
+      <c r="M42">
+        <v>9.309314310046357</v>
+      </c>
+      <c r="N42">
+        <v>64.30694977938343</v>
+      </c>
+      <c r="O42">
+        <v>125.2142099057482</v>
+      </c>
+      <c r="P42">
+        <v>198</v>
+      </c>
+      <c r="Q42">
+        <v>39</v>
+      </c>
+      <c r="R42">
+        <v>27</v>
+      </c>
+      <c r="S42">
+        <v>14.181</v>
       </c>
     </row>
   </sheetData>

</xml_diff>